<commit_message>
save 08 06 2026
</commit_message>
<xml_diff>
--- a/4 четверть_19_JavaScript_vite.xlsx
+++ b/4 четверть_19_JavaScript_vite.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0718363D-AD43-4C6C-BB6F-1F3BEAE625EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C59F3806-5763-42E3-B667-51E75176E8B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7080" yWindow="-19140" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9900" yWindow="-16290" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vite" sheetId="15" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="87">
   <si>
     <t>vite</t>
   </si>
@@ -1062,17 +1062,65 @@
   },</t>
     </r>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Создать проект vite + </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>vue3</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Создать проект </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>vite + [...]</t>
+    </r>
+  </si>
+  <si>
+    <t>npm create vue@latest</t>
+  </si>
+  <si>
+    <t>`https://github.com/vuejs/create-vue</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1271,9 +1319,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1281,47 +1329,47 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -1330,19 +1378,22 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1369,14 +1420,14 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>167999</xdr:colOff>
-      <xdr:row>47</xdr:row>
+      <xdr:row>48</xdr:row>
       <xdr:rowOff>58239</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1506668</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>4853941</xdr:rowOff>
+      <xdr:colOff>1502858</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>4857751</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1678,7 +1729,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:U107"/>
+  <dimension ref="A2:U108"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -1752,19 +1803,23 @@
       </c>
       <c r="S6" s="2"/>
     </row>
-    <row r="7" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B7" s="13" t="s">
-        <v>50</v>
-      </c>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B7" s="25"/>
       <c r="C7" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>51</v>
+        <v>85</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>86</v>
       </c>
       <c r="S7" s="2"/>
     </row>
     <row r="8" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>84</v>
+      </c>
       <c r="B8" s="2" t="s">
         <v>46</v>
       </c>
@@ -1773,405 +1828,414 @@
       </c>
       <c r="S8" s="2"/>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A9" s="18" t="s">
+    <row r="9" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="S9" s="2"/>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A10" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="S9" s="2"/>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2"/>
+      <c r="S10" s="2"/>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C11" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="S10" s="2"/>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A11" s="19" t="s">
+      <c r="S11" s="2"/>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A12" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="S11" s="2"/>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A12" s="20" t="s">
+      <c r="C12" s="16"/>
+      <c r="S12" s="2"/>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A13" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="13"/>
-      <c r="S12" s="2"/>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12" t="s">
+      <c r="C13" s="15"/>
+      <c r="D13" s="13"/>
+      <c r="S13" s="2"/>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A14" s="12"/>
+      <c r="B14" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C14" s="12" t="s">
         <v>8</v>
-      </c>
-      <c r="D13" s="10"/>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>29</v>
       </c>
       <c r="D14" s="10"/>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" s="10"/>
       <c r="B15" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>30</v>
+        <v>9</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>29</v>
       </c>
       <c r="D15" s="10"/>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" s="10"/>
       <c r="B16" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>31</v>
+        <v>10</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="D16" s="10"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
       <c r="B17" s="10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D17" s="10"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="10"/>
       <c r="B18" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D18" s="10"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="10"/>
       <c r="B19" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D19" s="10"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="10"/>
       <c r="B20" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D20" s="10"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="10"/>
       <c r="B21" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D21" s="10"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="10"/>
       <c r="B22" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D22" s="10"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="10"/>
       <c r="B23" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D23" s="10"/>
     </row>
-    <row r="24" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
       <c r="B24" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D24" s="10"/>
     </row>
-    <row r="25" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="10"/>
       <c r="B25" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+      <c r="D25" s="10"/>
+    </row>
+    <row r="26" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26" s="10"/>
       <c r="B26" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="D26" s="10"/>
+        <v>21</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="10"/>
       <c r="B27" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D27" s="10"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="10"/>
       <c r="B28" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D28" s="10"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="10"/>
       <c r="B29" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="D29" s="10"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="10"/>
       <c r="B30" s="10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D30" s="10"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="10"/>
-      <c r="B31" s="12" t="s">
+      <c r="B31" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D31" s="10"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="10"/>
+      <c r="B32" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="20" t="s">
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B32" s="10"/>
-      <c r="C32" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="D32" s="12" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A33" s="10"/>
       <c r="B33" s="10"/>
       <c r="C33" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="D33" s="10"/>
+        <v>7</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="34" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A34" s="10"/>
       <c r="B34" s="10"/>
       <c r="C34" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="D34" s="10"/>
+    </row>
+    <row r="35" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A35" s="10"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D34" s="10"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="22" t="s">
+      <c r="D35" s="10"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="23" t="s">
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="B36" s="10"/>
-      <c r="C36" s="1"/>
-      <c r="D36" s="10"/>
-    </row>
-    <row r="37" spans="1:4" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A37" s="10"/>
       <c r="B37" s="10"/>
-      <c r="C37" s="24" t="s">
+      <c r="C37" s="1"/>
+      <c r="D37" s="10"/>
+    </row>
+    <row r="38" spans="1:4" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A38" s="10"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="D37" s="10"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="23" t="s">
+      <c r="D38" s="10"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="B38" s="21"/>
-      <c r="C38" s="21"/>
-      <c r="D38" s="21"/>
-    </row>
-    <row r="39" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="21"/>
-      <c r="B39" s="21" t="s">
+      <c r="B39" s="21"/>
+      <c r="C39" s="21"/>
+      <c r="D39" s="21"/>
+    </row>
+    <row r="40" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="21"/>
+      <c r="B40" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="C39" s="21" t="s">
+      <c r="C40" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="D39" s="21"/>
-    </row>
-    <row r="40" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A40" s="21" t="s">
+      <c r="D40" s="21"/>
+    </row>
+    <row r="41" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A41" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="B40" s="21" t="s">
+      <c r="B41" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="C40" s="21" t="s">
+      <c r="C41" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D40" s="21"/>
-    </row>
-    <row r="41" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="21" t="s">
+      <c r="D41" s="21"/>
+    </row>
+    <row r="42" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="21" t="s">
         <v>63</v>
-      </c>
-      <c r="B41" s="21"/>
-      <c r="C41" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="D41" s="21"/>
-    </row>
-    <row r="42" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A42" s="21" t="s">
-        <v>65</v>
       </c>
       <c r="B42" s="21"/>
       <c r="C42" s="21" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D42" s="21"/>
     </row>
-    <row r="43" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A43" s="21" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B43" s="21"/>
       <c r="C43" s="21" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D43" s="21"/>
     </row>
-    <row r="44" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A44" s="21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B44" s="21"/>
       <c r="C44" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="D44" s="21"/>
+    </row>
+    <row r="45" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A45" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="B45" s="21"/>
+      <c r="C45" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="D44" s="21"/>
-    </row>
-    <row r="45" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A45" s="23" t="s">
+      <c r="D45" s="21"/>
+    </row>
+    <row r="46" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A46" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="B45" s="21" t="s">
+      <c r="B46" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="C45" s="21"/>
-      <c r="D45" s="10"/>
-    </row>
-    <row r="46" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="21" t="s">
+      <c r="C46" s="21"/>
+      <c r="D46" s="10"/>
+    </row>
+    <row r="47" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A47" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="B46" s="21"/>
-      <c r="C46" s="21" t="s">
+      <c r="B47" s="21"/>
+      <c r="C47" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="D46" s="10"/>
-    </row>
-    <row r="47" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A47" s="23" t="s">
+      <c r="D47" s="10"/>
+    </row>
+    <row r="48" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A48" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="B47" s="21" t="s">
+      <c r="B48" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="C47" s="21"/>
-      <c r="D47" s="21"/>
-    </row>
-    <row r="48" spans="1:4" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A48" s="21"/>
-      <c r="B48" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="C48" s="21" t="s">
-        <v>79</v>
-      </c>
+      <c r="C48" s="21"/>
       <c r="D48" s="21"/>
     </row>
-    <row r="49" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A49" s="21"/>
       <c r="B49" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="C49" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="D49" s="21"/>
+    </row>
+    <row r="50" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A50" s="21"/>
+      <c r="B50" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="C49" s="21" t="s">
+      <c r="C50" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="D49" s="21"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A50" s="10"/>
-      <c r="B50" s="10"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="10"/>
+      <c r="D50" s="21"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="10"/>
@@ -2515,8 +2579,14 @@
       <c r="C107" s="10"/>
       <c r="D107" s="10"/>
     </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A108" s="10"/>
+      <c r="B108" s="10"/>
+      <c r="C108" s="10"/>
+      <c r="D108" s="10"/>
+    </row>
   </sheetData>
-  <phoneticPr fontId="16" type="noConversion"/>
+  <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>

<commit_message>
save 15 07 2026
</commit_message>
<xml_diff>
--- a/4 четверть_19_JavaScript_vite.xlsx
+++ b/4 четверть_19_JavaScript_vite.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{251CF88E-FBC9-4741-AB0C-20012C812005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E0D2B5D-19E2-4D58-81D3-58322A654FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vite" sheetId="15" r:id="rId1"/>
-    <sheet name="env" sheetId="16" r:id="rId2"/>
+    <sheet name="Environment variables" sheetId="16" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="108">
   <si>
     <t>vite</t>
   </si>
@@ -705,21 +705,6 @@
   </si>
   <si>
     <t>plugins/env.js</t>
-  </si>
-  <si>
-    <t>const EnvPlugin = {
-  install(Vue) {
-    Vue.prototype.$env = {
-      isLocalProxy: import.meta.env.VITE_LOCALPROXY,
-      isElectronProxy: import.meta.env.VITE_ELECTRON_PROXY,
-      pathToBuild: import.meta.env.VITE_PAT_TO_BUILD,
-      apiProxy: import.meta.env.VITE_API_PROXY,
-      socketProxy: import.meta.env.VITE_SOCKET_PROXY,
-      fileLoaderPath: import.meta.env.VITE_FILE_LOAD,
-    }
-  }
-}
-export default EnvPlugin</t>
   </si>
   <si>
     <t>package.json</t>
@@ -1008,6 +993,46 @@
   </si>
   <si>
     <r>
+      <t xml:space="preserve">Создать проект vite + </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>vue3</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Создать проект </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>vite + [...]</t>
+    </r>
+  </si>
+  <si>
+    <t>npm create vue@latest</t>
+  </si>
+  <si>
+    <t>`https://github.com/vuejs/create-vue</t>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">scripts": {
     "dev": "vite --mode development",
     "build": "export NODE_OPTIONS=--openssl-legacy-provider &amp;&amp; vite build </t>
@@ -1055,8 +1080,30 @@
         <charset val="204"/>
         <scheme val="minor"/>
       </rPr>
+      <t xml:space="preserve">",
+    "electronbuilddev": "vite build </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>--mode electrondev</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>",
-    "electronbuilddev": "vite build --mode electrondev",
     "electronbuildprod": "vite build --mode electronprod",
     "electron": "electron .",
     "dist": "electron-builder --win --x64"
@@ -1065,7 +1112,31 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Создать проект vite + </t>
+      <t xml:space="preserve">const EnvPlugin = {
+  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>install</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(</t>
     </r>
     <r>
       <rPr>
@@ -1077,12 +1148,19 @@
         <charset val="204"/>
         <scheme val="minor"/>
       </rPr>
-      <t>vue3</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Создать проект </t>
+      <t>Vue</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">) {
+    </t>
     </r>
     <r>
       <rPr>
@@ -1094,26 +1172,669 @@
         <charset val="204"/>
         <scheme val="minor"/>
       </rPr>
-      <t>vite + [...]</t>
-    </r>
-  </si>
-  <si>
-    <t>npm create vue@latest</t>
-  </si>
-  <si>
-    <t>`https://github.com/vuejs/create-vue</t>
+      <t>Vue.prototype.$env</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = {
+      isLocalProxy: import.meta.env.VITE_LOCALPROXY,
+      isElectronProxy: import.meta.env.VITE_ELECTRON_PROXY,
+      pathToBuild: import.meta.env.VITE_PAT_TO_BUILD,
+      apiProxy: import.meta.env.VITE_API_PROXY,
+      socketProxy: import.meta.env.VITE_SOCKET_PROXY,
+      fileLoaderPath: import.meta.env.VITE_FILE_LOAD,
+    }
+  }
+}
+export default EnvPlugin</t>
+    </r>
+  </si>
+  <si>
+    <t>main.js</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">import </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>EnvPlugin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> from './plugins/env.js'
+Vue.use(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>EnvPlugin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>);</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">// plugins/env.js
+export default {
+  install(app) {
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>app.config.globalProperties.$env</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = {
+      isLocalProxy: import.meta.env.VITE_LOCALPROXY,
+      // ... остальные переменные
+    }
+  }
+}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">import </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>EnvPlugin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> from './plugins/env'
+const app = createApp(App)
+app.use(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>EnvPlugin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)
+app.mount('#app')</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Способ!</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> plugin</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Способ!</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Vite config</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>console.log(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>__API_URL__</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) // Работает везде</t>
+    </r>
+  </si>
+  <si>
+    <t>vite.config.js</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">export default defineConfig({
+  define: {
+    // Преобразуем env-переменные в константы (доступны везде)
+   </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> __API_URL__</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: JSON.stringify(process.env.VITE_API_PROXY),
+  }
+})</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Важные нюансы</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1 В Vite доступны ТОЛЬКО переменные с префиксом </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>VITE_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+2 Переменные окружения всегда </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>строки</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Способ!</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Composable</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">// composables/useEnv.js
+export const </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>useEnv</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = () =&gt; {
+  const </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>env</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = {
+    isLocalProxy: import.meta.env.VITE_LOCALPROXY === 'true',
+    isElectronProxy: import.meta.env.VITE_ELECTRON_PROXY === 'true',
+    pathToBuild: import.meta.env.VITE_PAT_TO_BUILD || '',
+    apiProxy: import.meta.env.VITE_API_PROXY || '',
+    socketProxy: import.meta.env.VITE_SOCKET_PROXY || '',
+    fileLoaderPath: import.meta.env.VITE_FILE_LOAD || '',
+    storagePublicUrl: import.meta.env.VITE_STORAGE_PUBLIC_URL || '',
+    nodeEnv: import.meta.env.VITE_NODE_ENV || 'development',
+  }
+  return </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>env</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+}</t>
+    </r>
+  </si>
+  <si>
+    <t>в компоненте</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">&lt;script setup&gt;
+import { </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>useEnv</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> } from '@/composables/useEnv'
+const { apiProxy, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>isLocalProxy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> } = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>useEnv()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+// Теперь isLocalProxy — это boolean, а не строка
+if (isLocalProxy) {
+  console.log('Работаем локально!')
+}
+&lt;/script&gt;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">import </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Vue</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> from 'vue';
+this.$http.post(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>this.$env.apiProxy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> + '/auth/login', {
+          username: this.username, 
+          password: hash, 
+          key: !this.username.isEmpty() &amp;&amp; !this.password.isEmpty() ? null : key, 
+          type: !this.username.isEmpty() &amp;&amp; !this.password.isEmpty() ? null : type,
+        })</t>
+    </r>
+  </si>
+  <si>
+    <t>Шаг 1</t>
+  </si>
+  <si>
+    <t>Шаг 2</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Доступ к переменным окружения в </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>vite.config.js</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Доступ к переменным окружения в </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>проекте</t>
+    </r>
+  </si>
+  <si>
+    <t>Шаг 3</t>
+  </si>
+  <si>
+    <t>Шаг 4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1279,7 +2000,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1316,6 +2037,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1328,9 +2055,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1338,47 +2065,47 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -1387,22 +2114,40 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1429,13 +2174,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>167999</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>58239</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>1502858</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>4857751</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1814,20 +2559,20 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B7" s="24"/>
       <c r="C7" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="S7" s="2"/>
     </row>
     <row r="8" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>46</v>
@@ -1839,7 +2584,7 @@
     </row>
     <row r="9" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B9" s="13" t="s">
         <v>50</v>
@@ -2217,7 +2962,7 @@
       <c r="D54" s="10"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="18" type="noConversion"/>
+  <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
@@ -2228,7 +2973,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:AA75"/>
+  <dimension ref="A2:AA86"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -2259,188 +3004,62 @@
     <col min="28" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="5"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="7"/>
-      <c r="G2" s="8"/>
-      <c r="P2" s="8"/>
-      <c r="Q2" s="8"/>
-      <c r="R2" s="8"/>
-      <c r="T2" s="9"/>
-      <c r="U2" s="8"/>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A2" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="C3" s="25" t="s">
+      <c r="A3" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="5"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="7"/>
+      <c r="G7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="T7" s="9"/>
+      <c r="U7" s="8"/>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="C8" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="S3" s="2"/>
-    </row>
-    <row r="4" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="22" t="s">
-        <v>76</v>
-      </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="10"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="1"/>
-      <c r="T4"/>
-      <c r="U4" s="2"/>
-      <c r="V4" s="1"/>
-      <c r="W4" s="1"/>
-      <c r="X4" s="1"/>
-      <c r="Y4" s="1"/>
-      <c r="Z4" s="1"/>
-      <c r="AA4" s="1"/>
-    </row>
-    <row r="5" spans="1:27" s="4" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="D5" s="10"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="1"/>
-      <c r="T5"/>
-      <c r="U5" s="2"/>
-      <c r="V5" s="1"/>
-      <c r="W5" s="1"/>
-      <c r="X5" s="1"/>
-      <c r="Y5" s="1"/>
-      <c r="Z5" s="1"/>
-      <c r="AA5" s="1"/>
-    </row>
-    <row r="6" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="22" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="1"/>
-      <c r="T6"/>
-      <c r="U6" s="2"/>
-      <c r="V6" s="1"/>
-      <c r="W6" s="1"/>
-      <c r="X6" s="1"/>
-      <c r="Y6" s="1"/>
-      <c r="Z6" s="1"/>
-      <c r="AA6" s="1"/>
-    </row>
-    <row r="7" spans="1:27" s="4" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="21"/>
-      <c r="B7" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="D7" s="21"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="1"/>
-      <c r="T7"/>
-      <c r="U7" s="2"/>
-      <c r="V7" s="1"/>
-      <c r="W7" s="1"/>
-      <c r="X7" s="1"/>
-      <c r="Y7" s="1"/>
-      <c r="Z7" s="1"/>
-      <c r="AA7" s="1"/>
-    </row>
-    <row r="8" spans="1:27" s="4" customFormat="1" ht="72" x14ac:dyDescent="0.3">
-      <c r="A8" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="C8" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="D8" s="21"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="1"/>
-      <c r="T8"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="1"/>
-      <c r="W8" s="1"/>
-      <c r="X8" s="1"/>
-      <c r="Y8" s="1"/>
-      <c r="Z8" s="1"/>
-      <c r="AA8" s="1"/>
-    </row>
-    <row r="9" spans="1:27" s="4" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="B9" s="21"/>
-      <c r="C9" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="D9" s="21"/>
+      <c r="S8" s="2"/>
+    </row>
+    <row r="9" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="10"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="10"/>
       <c r="F9" s="1"/>
       <c r="G9" s="2"/>
       <c r="H9" s="1"/>
@@ -2464,15 +3083,15 @@
       <c r="Z9" s="1"/>
       <c r="AA9" s="1"/>
     </row>
-    <row r="10" spans="1:27" s="4" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="D10" s="21"/>
+    <row r="10" spans="1:27" s="4" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="10"/>
+      <c r="B10" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="D10" s="10"/>
       <c r="F10" s="1"/>
       <c r="G10" s="2"/>
       <c r="H10" s="1"/>
@@ -2496,14 +3115,12 @@
       <c r="Z10" s="1"/>
       <c r="AA10" s="1"/>
     </row>
-    <row r="11" spans="1:27" s="4" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="21" t="s">
-        <v>67</v>
+    <row r="11" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="22" t="s">
+        <v>71</v>
       </c>
       <c r="B11" s="21"/>
-      <c r="C11" s="21" t="s">
-        <v>68</v>
-      </c>
+      <c r="C11" s="21"/>
       <c r="D11" s="21"/>
       <c r="F11" s="1"/>
       <c r="G11" s="2"/>
@@ -2528,13 +3145,13 @@
       <c r="Z11" s="1"/>
       <c r="AA11" s="1"/>
     </row>
-    <row r="12" spans="1:27" s="4" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="B12" s="21"/>
+    <row r="12" spans="1:27" s="4" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="21"/>
+      <c r="B12" s="21" t="s">
+        <v>59</v>
+      </c>
       <c r="C12" s="21" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D12" s="21"/>
       <c r="F12" s="1"/>
@@ -2560,15 +3177,17 @@
       <c r="Z12" s="1"/>
       <c r="AA12" s="1"/>
     </row>
-    <row r="13" spans="1:27" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="22" t="s">
-        <v>72</v>
+    <row r="13" spans="1:27" s="4" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+      <c r="A13" s="26" t="s">
+        <v>61</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="C13" s="21"/>
-      <c r="D13" s="10"/>
+        <v>58</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13" s="21"/>
       <c r="F13" s="1"/>
       <c r="G13" s="2"/>
       <c r="H13" s="1"/>
@@ -2592,15 +3211,15 @@
       <c r="Z13" s="1"/>
       <c r="AA13" s="1"/>
     </row>
-    <row r="14" spans="1:27" s="4" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:27" s="4" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="21" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="B14" s="21"/>
       <c r="C14" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="D14" s="10"/>
+        <v>64</v>
+      </c>
+      <c r="D14" s="21"/>
       <c r="F14" s="1"/>
       <c r="G14" s="2"/>
       <c r="H14" s="1"/>
@@ -2624,14 +3243,14 @@
       <c r="Z14" s="1"/>
       <c r="AA14" s="1"/>
     </row>
-    <row r="15" spans="1:27" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="C15" s="21"/>
+    <row r="15" spans="1:27" s="4" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21" t="s">
+        <v>66</v>
+      </c>
       <c r="D15" s="21"/>
       <c r="F15" s="1"/>
       <c r="G15" s="2"/>
@@ -2656,13 +3275,13 @@
       <c r="Z15" s="1"/>
       <c r="AA15" s="1"/>
     </row>
-    <row r="16" spans="1:27" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="21"/>
-      <c r="B16" s="21" t="s">
-        <v>78</v>
-      </c>
+    <row r="16" spans="1:27" s="4" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="B16" s="21"/>
       <c r="C16" s="21" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="D16" s="21"/>
       <c r="F16" s="1"/>
@@ -2688,13 +3307,13 @@
       <c r="Z16" s="1"/>
       <c r="AA16" s="1"/>
     </row>
-    <row r="17" spans="1:27" s="4" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="21"/>
-      <c r="B17" s="21" t="s">
-        <v>80</v>
-      </c>
+    <row r="17" spans="1:27" s="4" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="21"/>
       <c r="C17" s="21" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="D17" s="21"/>
       <c r="F17" s="1"/>
@@ -2720,11 +3339,15 @@
       <c r="Z17" s="1"/>
       <c r="AA17" s="1"/>
     </row>
-    <row r="18" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
+    <row r="18" spans="1:27" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
       <c r="F18" s="1"/>
       <c r="G18" s="2"/>
       <c r="H18" s="1"/>
@@ -2748,67 +3371,40 @@
       <c r="Z18" s="1"/>
       <c r="AA18" s="1"/>
     </row>
-    <row r="19" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19" s="2"/>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="2"/>
-      <c r="S19" s="1"/>
-      <c r="T19"/>
-      <c r="U19" s="2"/>
-      <c r="V19" s="1"/>
-      <c r="W19" s="1"/>
-      <c r="X19" s="1"/>
-      <c r="Y19" s="1"/>
-      <c r="Z19" s="1"/>
-      <c r="AA19" s="1"/>
-    </row>
-    <row r="20" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="10"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
-      <c r="P20" s="2"/>
-      <c r="Q20" s="2"/>
-      <c r="R20" s="2"/>
-      <c r="S20" s="1"/>
-      <c r="T20"/>
-      <c r="U20" s="2"/>
-      <c r="V20" s="1"/>
-      <c r="W20" s="1"/>
-      <c r="X20" s="1"/>
-      <c r="Y20" s="1"/>
-      <c r="Z20" s="1"/>
-      <c r="AA20" s="1"/>
+    <row r="19" spans="1:27" s="21" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="B19" s="28" t="s">
+        <v>99</v>
+      </c>
+      <c r="C19" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="E19" s="31"/>
+    </row>
+    <row r="20" spans="1:27" s="21" customFormat="1" ht="216" x14ac:dyDescent="0.3">
+      <c r="B20" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="C20" s="27" t="s">
+        <v>98</v>
+      </c>
+      <c r="E20" s="31"/>
     </row>
     <row r="21" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="10"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
+      <c r="A21" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="B21" s="28" t="s">
+        <v>99</v>
+      </c>
+      <c r="C21" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="D21" s="28" t="s">
+        <v>54</v>
+      </c>
       <c r="F21" s="1"/>
       <c r="G21" s="2"/>
       <c r="H21" s="1"/>
@@ -2832,11 +3428,19 @@
       <c r="Z21" s="1"/>
       <c r="AA21" s="1"/>
     </row>
-    <row r="22" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="10"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
+    <row r="22" spans="1:27" s="4" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="C22" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="D22" s="27" t="s">
+        <v>86</v>
+      </c>
       <c r="F22" s="1"/>
       <c r="G22" s="2"/>
       <c r="H22" s="1"/>
@@ -2860,11 +3464,17 @@
       <c r="Z22" s="1"/>
       <c r="AA22" s="1"/>
     </row>
-    <row r="23" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
+    <row r="23" spans="1:27" s="4" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+      <c r="A23" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="D23" s="27" t="s">
+        <v>88</v>
+      </c>
       <c r="F23" s="1"/>
       <c r="G23" s="2"/>
       <c r="H23" s="1"/>
@@ -2889,10 +3499,12 @@
       <c r="AA23" s="1"/>
     </row>
     <row r="24" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="10"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
+      <c r="A24" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="B24" s="21"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
       <c r="F24" s="1"/>
       <c r="G24" s="2"/>
       <c r="H24" s="1"/>
@@ -2916,11 +3528,17 @@
       <c r="Z24" s="1"/>
       <c r="AA24" s="1"/>
     </row>
-    <row r="25" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="10"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
+    <row r="25" spans="1:27" s="4" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A25" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="B25" s="21"/>
+      <c r="C25" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="D25" s="27" t="s">
+        <v>93</v>
+      </c>
       <c r="F25" s="1"/>
       <c r="G25" s="2"/>
       <c r="H25" s="1"/>
@@ -2944,11 +3562,15 @@
       <c r="Z25" s="1"/>
       <c r="AA25" s="1"/>
     </row>
-    <row r="26" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="10"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
+    <row r="26" spans="1:27" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
       <c r="F26" s="1"/>
       <c r="G26" s="2"/>
       <c r="H26" s="1"/>
@@ -2972,11 +3594,15 @@
       <c r="Z26" s="1"/>
       <c r="AA26" s="1"/>
     </row>
-    <row r="27" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="10"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
+    <row r="27" spans="1:27" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="21"/>
+      <c r="B27" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="C27" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="D27" s="21"/>
       <c r="F27" s="1"/>
       <c r="G27" s="2"/>
       <c r="H27" s="1"/>
@@ -3000,11 +3626,15 @@
       <c r="Z27" s="1"/>
       <c r="AA27" s="1"/>
     </row>
-    <row r="28" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="10"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
+    <row r="28" spans="1:27" s="4" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="21"/>
+      <c r="B28" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="D28" s="21"/>
       <c r="F28" s="1"/>
       <c r="G28" s="2"/>
       <c r="H28" s="1"/>
@@ -4344,7 +4974,316 @@
       <c r="Z75" s="1"/>
       <c r="AA75" s="1"/>
     </row>
+    <row r="76" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="10"/>
+      <c r="B76" s="10"/>
+      <c r="C76" s="10"/>
+      <c r="D76" s="10"/>
+      <c r="F76" s="1"/>
+      <c r="G76" s="2"/>
+      <c r="H76" s="1"/>
+      <c r="I76" s="1"/>
+      <c r="J76" s="1"/>
+      <c r="K76" s="1"/>
+      <c r="L76" s="1"/>
+      <c r="M76" s="1"/>
+      <c r="N76" s="1"/>
+      <c r="O76" s="1"/>
+      <c r="P76" s="2"/>
+      <c r="Q76" s="2"/>
+      <c r="R76" s="2"/>
+      <c r="S76" s="1"/>
+      <c r="T76"/>
+      <c r="U76" s="2"/>
+      <c r="V76" s="1"/>
+      <c r="W76" s="1"/>
+      <c r="X76" s="1"/>
+      <c r="Y76" s="1"/>
+      <c r="Z76" s="1"/>
+      <c r="AA76" s="1"/>
+    </row>
+    <row r="77" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="10"/>
+      <c r="B77" s="10"/>
+      <c r="C77" s="10"/>
+      <c r="D77" s="10"/>
+      <c r="F77" s="1"/>
+      <c r="G77" s="2"/>
+      <c r="H77" s="1"/>
+      <c r="I77" s="1"/>
+      <c r="J77" s="1"/>
+      <c r="K77" s="1"/>
+      <c r="L77" s="1"/>
+      <c r="M77" s="1"/>
+      <c r="N77" s="1"/>
+      <c r="O77" s="1"/>
+      <c r="P77" s="2"/>
+      <c r="Q77" s="2"/>
+      <c r="R77" s="2"/>
+      <c r="S77" s="1"/>
+      <c r="T77"/>
+      <c r="U77" s="2"/>
+      <c r="V77" s="1"/>
+      <c r="W77" s="1"/>
+      <c r="X77" s="1"/>
+      <c r="Y77" s="1"/>
+      <c r="Z77" s="1"/>
+      <c r="AA77" s="1"/>
+    </row>
+    <row r="78" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="10"/>
+      <c r="B78" s="10"/>
+      <c r="C78" s="10"/>
+      <c r="D78" s="10"/>
+      <c r="F78" s="1"/>
+      <c r="G78" s="2"/>
+      <c r="H78" s="1"/>
+      <c r="I78" s="1"/>
+      <c r="J78" s="1"/>
+      <c r="K78" s="1"/>
+      <c r="L78" s="1"/>
+      <c r="M78" s="1"/>
+      <c r="N78" s="1"/>
+      <c r="O78" s="1"/>
+      <c r="P78" s="2"/>
+      <c r="Q78" s="2"/>
+      <c r="R78" s="2"/>
+      <c r="S78" s="1"/>
+      <c r="T78"/>
+      <c r="U78" s="2"/>
+      <c r="V78" s="1"/>
+      <c r="W78" s="1"/>
+      <c r="X78" s="1"/>
+      <c r="Y78" s="1"/>
+      <c r="Z78" s="1"/>
+      <c r="AA78" s="1"/>
+    </row>
+    <row r="79" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="10"/>
+      <c r="B79" s="10"/>
+      <c r="C79" s="10"/>
+      <c r="D79" s="10"/>
+      <c r="F79" s="1"/>
+      <c r="G79" s="2"/>
+      <c r="H79" s="1"/>
+      <c r="I79" s="1"/>
+      <c r="J79" s="1"/>
+      <c r="K79" s="1"/>
+      <c r="L79" s="1"/>
+      <c r="M79" s="1"/>
+      <c r="N79" s="1"/>
+      <c r="O79" s="1"/>
+      <c r="P79" s="2"/>
+      <c r="Q79" s="2"/>
+      <c r="R79" s="2"/>
+      <c r="S79" s="1"/>
+      <c r="T79"/>
+      <c r="U79" s="2"/>
+      <c r="V79" s="1"/>
+      <c r="W79" s="1"/>
+      <c r="X79" s="1"/>
+      <c r="Y79" s="1"/>
+      <c r="Z79" s="1"/>
+      <c r="AA79" s="1"/>
+    </row>
+    <row r="80" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="10"/>
+      <c r="B80" s="10"/>
+      <c r="C80" s="10"/>
+      <c r="D80" s="10"/>
+      <c r="F80" s="1"/>
+      <c r="G80" s="2"/>
+      <c r="H80" s="1"/>
+      <c r="I80" s="1"/>
+      <c r="J80" s="1"/>
+      <c r="K80" s="1"/>
+      <c r="L80" s="1"/>
+      <c r="M80" s="1"/>
+      <c r="N80" s="1"/>
+      <c r="O80" s="1"/>
+      <c r="P80" s="2"/>
+      <c r="Q80" s="2"/>
+      <c r="R80" s="2"/>
+      <c r="S80" s="1"/>
+      <c r="T80"/>
+      <c r="U80" s="2"/>
+      <c r="V80" s="1"/>
+      <c r="W80" s="1"/>
+      <c r="X80" s="1"/>
+      <c r="Y80" s="1"/>
+      <c r="Z80" s="1"/>
+      <c r="AA80" s="1"/>
+    </row>
+    <row r="81" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="10"/>
+      <c r="B81" s="10"/>
+      <c r="C81" s="10"/>
+      <c r="D81" s="10"/>
+      <c r="F81" s="1"/>
+      <c r="G81" s="2"/>
+      <c r="H81" s="1"/>
+      <c r="I81" s="1"/>
+      <c r="J81" s="1"/>
+      <c r="K81" s="1"/>
+      <c r="L81" s="1"/>
+      <c r="M81" s="1"/>
+      <c r="N81" s="1"/>
+      <c r="O81" s="1"/>
+      <c r="P81" s="2"/>
+      <c r="Q81" s="2"/>
+      <c r="R81" s="2"/>
+      <c r="S81" s="1"/>
+      <c r="T81"/>
+      <c r="U81" s="2"/>
+      <c r="V81" s="1"/>
+      <c r="W81" s="1"/>
+      <c r="X81" s="1"/>
+      <c r="Y81" s="1"/>
+      <c r="Z81" s="1"/>
+      <c r="AA81" s="1"/>
+    </row>
+    <row r="82" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="10"/>
+      <c r="B82" s="10"/>
+      <c r="C82" s="10"/>
+      <c r="D82" s="10"/>
+      <c r="F82" s="1"/>
+      <c r="G82" s="2"/>
+      <c r="H82" s="1"/>
+      <c r="I82" s="1"/>
+      <c r="J82" s="1"/>
+      <c r="K82" s="1"/>
+      <c r="L82" s="1"/>
+      <c r="M82" s="1"/>
+      <c r="N82" s="1"/>
+      <c r="O82" s="1"/>
+      <c r="P82" s="2"/>
+      <c r="Q82" s="2"/>
+      <c r="R82" s="2"/>
+      <c r="S82" s="1"/>
+      <c r="T82"/>
+      <c r="U82" s="2"/>
+      <c r="V82" s="1"/>
+      <c r="W82" s="1"/>
+      <c r="X82" s="1"/>
+      <c r="Y82" s="1"/>
+      <c r="Z82" s="1"/>
+      <c r="AA82" s="1"/>
+    </row>
+    <row r="83" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="10"/>
+      <c r="B83" s="10"/>
+      <c r="C83" s="10"/>
+      <c r="D83" s="10"/>
+      <c r="F83" s="1"/>
+      <c r="G83" s="2"/>
+      <c r="H83" s="1"/>
+      <c r="I83" s="1"/>
+      <c r="J83" s="1"/>
+      <c r="K83" s="1"/>
+      <c r="L83" s="1"/>
+      <c r="M83" s="1"/>
+      <c r="N83" s="1"/>
+      <c r="O83" s="1"/>
+      <c r="P83" s="2"/>
+      <c r="Q83" s="2"/>
+      <c r="R83" s="2"/>
+      <c r="S83" s="1"/>
+      <c r="T83"/>
+      <c r="U83" s="2"/>
+      <c r="V83" s="1"/>
+      <c r="W83" s="1"/>
+      <c r="X83" s="1"/>
+      <c r="Y83" s="1"/>
+      <c r="Z83" s="1"/>
+      <c r="AA83" s="1"/>
+    </row>
+    <row r="84" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="10"/>
+      <c r="B84" s="10"/>
+      <c r="C84" s="10"/>
+      <c r="D84" s="10"/>
+      <c r="F84" s="1"/>
+      <c r="G84" s="2"/>
+      <c r="H84" s="1"/>
+      <c r="I84" s="1"/>
+      <c r="J84" s="1"/>
+      <c r="K84" s="1"/>
+      <c r="L84" s="1"/>
+      <c r="M84" s="1"/>
+      <c r="N84" s="1"/>
+      <c r="O84" s="1"/>
+      <c r="P84" s="2"/>
+      <c r="Q84" s="2"/>
+      <c r="R84" s="2"/>
+      <c r="S84" s="1"/>
+      <c r="T84"/>
+      <c r="U84" s="2"/>
+      <c r="V84" s="1"/>
+      <c r="W84" s="1"/>
+      <c r="X84" s="1"/>
+      <c r="Y84" s="1"/>
+      <c r="Z84" s="1"/>
+      <c r="AA84" s="1"/>
+    </row>
+    <row r="85" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="10"/>
+      <c r="B85" s="10"/>
+      <c r="C85" s="10"/>
+      <c r="D85" s="10"/>
+      <c r="F85" s="1"/>
+      <c r="G85" s="2"/>
+      <c r="H85" s="1"/>
+      <c r="I85" s="1"/>
+      <c r="J85" s="1"/>
+      <c r="K85" s="1"/>
+      <c r="L85" s="1"/>
+      <c r="M85" s="1"/>
+      <c r="N85" s="1"/>
+      <c r="O85" s="1"/>
+      <c r="P85" s="2"/>
+      <c r="Q85" s="2"/>
+      <c r="R85" s="2"/>
+      <c r="S85" s="1"/>
+      <c r="T85"/>
+      <c r="U85" s="2"/>
+      <c r="V85" s="1"/>
+      <c r="W85" s="1"/>
+      <c r="X85" s="1"/>
+      <c r="Y85" s="1"/>
+      <c r="Z85" s="1"/>
+      <c r="AA85" s="1"/>
+    </row>
+    <row r="86" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="10"/>
+      <c r="B86" s="10"/>
+      <c r="C86" s="10"/>
+      <c r="D86" s="10"/>
+      <c r="F86" s="1"/>
+      <c r="G86" s="2"/>
+      <c r="H86" s="1"/>
+      <c r="I86" s="1"/>
+      <c r="J86" s="1"/>
+      <c r="K86" s="1"/>
+      <c r="L86" s="1"/>
+      <c r="M86" s="1"/>
+      <c r="N86" s="1"/>
+      <c r="O86" s="1"/>
+      <c r="P86" s="2"/>
+      <c r="Q86" s="2"/>
+      <c r="R86" s="2"/>
+      <c r="S86" s="1"/>
+      <c r="T86"/>
+      <c r="U86" s="2"/>
+      <c r="V86" s="1"/>
+      <c r="W86" s="1"/>
+      <c r="X86" s="1"/>
+      <c r="Y86" s="1"/>
+      <c r="Z86" s="1"/>
+      <c r="AA86" s="1"/>
+    </row>
   </sheetData>
+  <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>

<commit_message>
save 17 07 2026
</commit_message>
<xml_diff>
--- a/4 четверть_19_JavaScript_vite.xlsx
+++ b/4 четверть_19_JavaScript_vite.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E0D2B5D-19E2-4D58-81D3-58322A654FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F81B1623-4372-43AF-BD68-500A2C1FFFDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vite" sheetId="15" r:id="rId1"/>
@@ -219,67 +219,6 @@
   </si>
   <si>
     <t>template названия</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">npm create vite@latest </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>my-vue-app</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>--</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> --template </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>vue</t>
-    </r>
   </si>
   <si>
     <r>
@@ -1816,17 +1755,153 @@
   <si>
     <t>Шаг 4</t>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">npm create vite@latest </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>my-vue-app</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>--</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> --template </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>vue</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> //my-vue-app folder</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">npm create vite@latest </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">-- --template vue </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> //current directory</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1999,6 +2074,14 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -2055,7 +2138,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2065,47 +2148,47 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="15" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -2114,40 +2197,40 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2540,17 +2623,17 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" s="17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C5" s="2"/>
       <c r="S5" s="2"/>
     </row>
     <row r="6" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>45</v>
@@ -2559,47 +2642,47 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B7" s="24"/>
       <c r="C7" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D7" s="24" t="s">
         <v>83</v>
-      </c>
-      <c r="D7" s="24" t="s">
-        <v>84</v>
       </c>
       <c r="S7" s="2"/>
     </row>
     <row r="8" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>46</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="S8" s="2"/>
     </row>
     <row r="9" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B9" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D9" s="13" t="s">
         <v>50</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>51</v>
       </c>
       <c r="S9" s="2"/>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" s="18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C10" s="2"/>
       <c r="S10" s="2"/>
@@ -2607,16 +2690,16 @@
     <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S11" s="2"/>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C12" s="16"/>
       <c r="S12" s="2"/>
@@ -2962,7 +3045,7 @@
       <c r="D54" s="10"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="19" type="noConversion"/>
+  <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
@@ -3006,34 +3089,34 @@
   <sheetData>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:27" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:27" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="29" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -3049,13 +3132,13 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="C8" s="25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="S8" s="2"/>
     </row>
     <row r="9" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="1"/>
@@ -3086,10 +3169,10 @@
     <row r="10" spans="1:27" s="4" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A10" s="10"/>
       <c r="B10" s="27" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D10" s="10"/>
       <c r="F10" s="1"/>
@@ -3117,7 +3200,7 @@
     </row>
     <row r="11" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B11" s="21"/>
       <c r="C11" s="21"/>
@@ -3148,10 +3231,10 @@
     <row r="12" spans="1:27" s="4" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="21"/>
       <c r="B12" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="21" t="s">
         <v>59</v>
-      </c>
-      <c r="C12" s="21" t="s">
-        <v>60</v>
       </c>
       <c r="D12" s="21"/>
       <c r="F12" s="1"/>
@@ -3179,13 +3262,13 @@
     </row>
     <row r="13" spans="1:27" s="4" customFormat="1" ht="72" x14ac:dyDescent="0.3">
       <c r="A13" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" s="21" t="s">
         <v>61</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="C13" s="21" t="s">
-        <v>62</v>
       </c>
       <c r="D13" s="21"/>
       <c r="F13" s="1"/>
@@ -3213,11 +3296,11 @@
     </row>
     <row r="14" spans="1:27" s="4" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B14" s="21"/>
       <c r="C14" s="21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D14" s="21"/>
       <c r="F14" s="1"/>
@@ -3245,11 +3328,11 @@
     </row>
     <row r="15" spans="1:27" s="4" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B15" s="21"/>
       <c r="C15" s="21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D15" s="21"/>
       <c r="F15" s="1"/>
@@ -3277,11 +3360,11 @@
     </row>
     <row r="16" spans="1:27" s="4" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B16" s="21"/>
       <c r="C16" s="21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D16" s="21"/>
       <c r="F16" s="1"/>
@@ -3309,11 +3392,11 @@
     </row>
     <row r="17" spans="1:27" s="4" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A17" s="21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B17" s="21"/>
       <c r="C17" s="21" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D17" s="21"/>
       <c r="F17" s="1"/>
@@ -3341,10 +3424,10 @@
     </row>
     <row r="18" spans="1:27" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="21" t="s">
         <v>72</v>
-      </c>
-      <c r="B18" s="21" t="s">
-        <v>73</v>
       </c>
       <c r="C18" s="21"/>
       <c r="D18" s="21"/>
@@ -3373,37 +3456,37 @@
     </row>
     <row r="19" spans="1:27" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="30" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B19" s="28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C19" s="28" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E19" s="31"/>
     </row>
     <row r="20" spans="1:27" s="21" customFormat="1" ht="216" x14ac:dyDescent="0.3">
       <c r="B20" s="27" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C20" s="27" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E20" s="31"/>
     </row>
     <row r="21" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="30" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B21" s="28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C21" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="D21" s="28" t="s">
         <v>53</v>
-      </c>
-      <c r="D21" s="28" t="s">
-        <v>54</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="2"/>
@@ -3430,16 +3513,16 @@
     </row>
     <row r="22" spans="1:27" s="4" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A22" s="21" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B22" s="27" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D22" s="27" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="2"/>
@@ -3466,14 +3549,14 @@
     </row>
     <row r="23" spans="1:27" s="4" customFormat="1" ht="72" x14ac:dyDescent="0.3">
       <c r="A23" s="27" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B23" s="27"/>
       <c r="C23" s="27" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="2"/>
@@ -3500,7 +3583,7 @@
     </row>
     <row r="24" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="30" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B24" s="21"/>
       <c r="C24" s="27"/>
@@ -3530,14 +3613,14 @@
     </row>
     <row r="25" spans="1:27" s="4" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A25" s="27" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B25" s="21"/>
       <c r="C25" s="27" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D25" s="27" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="2"/>
@@ -3564,10 +3647,10 @@
     </row>
     <row r="26" spans="1:27" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C26" s="21"/>
       <c r="D26" s="21"/>
@@ -3597,10 +3680,10 @@
     <row r="27" spans="1:27" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A27" s="21"/>
       <c r="B27" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="C27" s="21" t="s">
         <v>77</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>78</v>
       </c>
       <c r="D27" s="21"/>
       <c r="F27" s="1"/>
@@ -3629,10 +3712,10 @@
     <row r="28" spans="1:27" s="4" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A28" s="21"/>
       <c r="B28" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="C28" s="21" t="s">
         <v>79</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>80</v>
       </c>
       <c r="D28" s="21"/>
       <c r="F28" s="1"/>
@@ -5283,7 +5366,7 @@
       <c r="AA86" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="19" type="noConversion"/>
+  <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>